<commit_message>
Add GO term analysis for day0 comparisons
</commit_message>
<xml_diff>
--- a/Output_plot/Apheresis_Day0vsControl_Day0_Deg_Up.xlsx
+++ b/Output_plot/Apheresis_Day0vsControl_Day0_Deg_Up.xlsx
@@ -394,526 +394,526 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ANP32A</t>
+          <t>NLRP2</t>
         </is>
       </c>
       <c r="B2">
-        <v>17.771</v>
+        <v>1.363754197653561</v>
       </c>
       <c r="C2">
-        <v>78.43294444444444</v>
+        <v>3.681423226082345</v>
       </c>
       <c r="D2">
-        <v>7.53276118430309</v>
+        <v>10.63776249380159</v>
       </c>
       <c r="E2">
-        <v>3.348079469281519E-06</v>
+        <v>1.524010458868847E-07</v>
       </c>
       <c r="F2">
-        <v>0.009737331123160419</v>
+        <v>0.0001108082604469224</v>
       </c>
       <c r="G2">
-        <v>2.049054363001395</v>
+        <v>7.837179935353091</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>TNFRSF17</t>
         </is>
       </c>
       <c r="B3">
-        <v>4.459333333333331</v>
+        <v>1.481747535822066</v>
       </c>
       <c r="C3">
-        <v>4.354833333333334</v>
+        <v>3.347270897334747</v>
       </c>
       <c r="D3">
-        <v>7.042385109021979</v>
+        <v>9.406120026756971</v>
       </c>
       <c r="E3">
-        <v>7.002949738965982E-06</v>
+        <v>5.898368617592659E-07</v>
       </c>
       <c r="F3">
-        <v>0.01527518411811955</v>
+        <v>0.0002769788066027396</v>
       </c>
       <c r="G3">
-        <v>1.707727332339468</v>
+        <v>6.570633597536797</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>THOC7</t>
+          <t>IGHV4.28</t>
         </is>
       </c>
       <c r="B4">
-        <v>10.56033333333334</v>
+        <v>1.20326419772433</v>
       </c>
       <c r="C4">
-        <v>28.78922222222222</v>
+        <v>4.781214558701351</v>
       </c>
       <c r="D4">
-        <v>6.69801185411521</v>
+        <v>8.948592624894104</v>
       </c>
       <c r="E4">
-        <v>1.198202762940756E-05</v>
+        <v>1.010433220938109E-06</v>
       </c>
       <c r="F4">
-        <v>0.01539295469995395</v>
+        <v>0.0003431099972348794</v>
       </c>
       <c r="G4">
-        <v>1.446814970597404</v>
+        <v>6.058300732164468</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TPI1</t>
+          <t>IGLV10.54</t>
         </is>
       </c>
       <c r="B5">
-        <v>42.83666666666666</v>
+        <v>1.647963420898776</v>
       </c>
       <c r="C5">
-        <v>131.0269444444444</v>
+        <v>5.646927181517103</v>
       </c>
       <c r="D5">
-        <v>6.424914660668504</v>
+        <v>8.309156666591697</v>
       </c>
       <c r="E5">
-        <v>1.855423467405756E-05</v>
+        <v>2.222176305366474E-06</v>
       </c>
       <c r="F5">
-        <v>0.01539295469995395</v>
+        <v>0.0005599633812095687</v>
       </c>
       <c r="G5">
-        <v>1.226630556315226</v>
+        <v>5.300619024594082</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PACSIN2</t>
+          <t>IGHG1</t>
         </is>
       </c>
       <c r="B6">
-        <v>5.669000000000001</v>
+        <v>1.85469940735972</v>
       </c>
       <c r="C6">
-        <v>14.71888888888889</v>
+        <v>9.004411904203067</v>
       </c>
       <c r="D6">
-        <v>6.419749703527456</v>
+        <v>8.302021190446441</v>
       </c>
       <c r="E6">
-        <v>1.871015673929048E-05</v>
+        <v>2.242359682315317E-06</v>
       </c>
       <c r="F6">
-        <v>0.01539295469995395</v>
+        <v>0.0005599633812095687</v>
       </c>
       <c r="G6">
-        <v>1.222349328044334</v>
+        <v>5.291878222537892</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PSMC3</t>
+          <t>CPT1B</t>
         </is>
       </c>
       <c r="B7">
-        <v>8.671000000000005</v>
+        <v>1.427373673231409</v>
       </c>
       <c r="C7">
-        <v>39.265</v>
+        <v>5.485182691527275</v>
       </c>
       <c r="D7">
-        <v>6.397220112664663</v>
+        <v>7.986442412187348</v>
       </c>
       <c r="E7">
-        <v>1.9406590452664E-05</v>
+        <v>3.363904596775141E-06</v>
       </c>
       <c r="F7">
-        <v>0.01539295469995395</v>
+        <v>0.0006052483465494858</v>
       </c>
       <c r="G7">
-        <v>1.203623001756926</v>
+        <v>4.898762459077308</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BRK1</t>
+          <t>IGHV1.2</t>
         </is>
       </c>
       <c r="B8">
-        <v>19.27933333333334</v>
+        <v>1.302232123990865</v>
       </c>
       <c r="C8">
-        <v>67.51950000000001</v>
+        <v>8.337567356638337</v>
       </c>
       <c r="D8">
-        <v>6.288274949591982</v>
+        <v>7.962974222233773</v>
       </c>
       <c r="E8">
-        <v>2.318077389614107E-05</v>
+        <v>3.468471899997053E-06</v>
       </c>
       <c r="F8">
-        <v>0.01621659213319319</v>
+        <v>0.0006052483465494858</v>
       </c>
       <c r="G8">
-        <v>1.111877339614087</v>
+        <v>4.869010919693912</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SARNP</t>
+          <t>RRM2</t>
         </is>
       </c>
       <c r="B9">
-        <v>9.699999999999999</v>
+        <v>1.084458683001281</v>
       </c>
       <c r="C9">
-        <v>34.9265</v>
+        <v>1.933747572376567</v>
       </c>
       <c r="D9">
-        <v>5.926631786137357</v>
+        <v>7.299302797920486</v>
       </c>
       <c r="E9">
-        <v>4.230959300339541E-05</v>
+        <v>8.468477585845492E-06</v>
       </c>
       <c r="F9">
-        <v>0.02185602114763466</v>
+        <v>0.001107443527125249</v>
       </c>
       <c r="G9">
-        <v>0.7928448089659357</v>
+        <v>3.996962266311967</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MTHFS</t>
+          <t>IGKV1.27</t>
         </is>
       </c>
       <c r="B10">
-        <v>4.142999999999999</v>
+        <v>1.282615759368759</v>
       </c>
       <c r="C10">
-        <v>5.431277777777777</v>
+        <v>7.836391093946304</v>
       </c>
       <c r="D10">
-        <v>5.9227935039849</v>
+        <v>7.296268766826409</v>
       </c>
       <c r="E10">
-        <v>4.258479765155177E-05</v>
+        <v>8.504150867322831E-06</v>
       </c>
       <c r="F10">
-        <v>0.02185602114763466</v>
+        <v>0.001107443527125249</v>
       </c>
       <c r="G10">
-        <v>0.7893369730020954</v>
+        <v>3.992836444546472</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PGM2</t>
+          <t>JCHAIN</t>
         </is>
       </c>
       <c r="B11">
-        <v>2.646666666666665</v>
+        <v>1.129670093090444</v>
       </c>
       <c r="C11">
-        <v>9.506833333333335</v>
+        <v>8.714490678241875</v>
       </c>
       <c r="D11">
-        <v>5.809827574924263</v>
+        <v>6.904048621968495</v>
       </c>
       <c r="E11">
-        <v>5.158511157280331E-05</v>
+        <v>1.478735729365778E-05</v>
       </c>
       <c r="F11">
-        <v>0.02309134726163446</v>
+        <v>0.001612746154839552</v>
       </c>
       <c r="G11">
-        <v>0.6849299221717136</v>
+        <v>3.448473255088047</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>H2AFZ</t>
+          <t>IGKV2.24</t>
         </is>
       </c>
       <c r="B12">
-        <v>15.80800000000002</v>
+        <v>1.048163990022892</v>
       </c>
       <c r="C12">
-        <v>73.86922222222223</v>
+        <v>6.551366337456438</v>
       </c>
       <c r="D12">
-        <v>5.604000325769774</v>
+        <v>6.877481519490812</v>
       </c>
       <c r="E12">
-        <v>7.348933967245097E-05</v>
+        <v>1.536294972282234E-05</v>
       </c>
       <c r="F12">
-        <v>0.02787802124531021</v>
+        <v>0.001634655321117377</v>
       </c>
       <c r="G12">
-        <v>0.4888349913202452</v>
+        <v>3.410802306915465</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ATP6V1E1</t>
+          <t>FP565260.1</t>
         </is>
       </c>
       <c r="B13">
-        <v>8.196333333333335</v>
+        <v>1.072231368770614</v>
       </c>
       <c r="C13">
-        <v>43.05688888888888</v>
+        <v>3.001295704228615</v>
       </c>
       <c r="D13">
-        <v>5.479083462282585</v>
+        <v>6.407605006166793</v>
       </c>
       <c r="E13">
-        <v>9.135802768430965E-05</v>
+        <v>3.06532697399585E-05</v>
       </c>
       <c r="F13">
-        <v>0.03065764582867699</v>
+        <v>0.0023056015386305</v>
       </c>
       <c r="G13">
-        <v>0.3660873797474551</v>
+        <v>2.727463067264405</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MYL12B</t>
+          <t>IGHV3.72</t>
         </is>
       </c>
       <c r="B14">
-        <v>26.5686666666667</v>
+        <v>1.597820200652561</v>
       </c>
       <c r="C14">
-        <v>121.6562222222222</v>
+        <v>5.468218355916342</v>
       </c>
       <c r="D14">
-        <v>5.195612855841769</v>
+        <v>6.076374520569526</v>
       </c>
       <c r="E14">
-        <v>0.0001508977657018373</v>
+        <v>5.078610764834027E-05</v>
       </c>
       <c r="F14">
-        <v>0.03558332447969002</v>
+        <v>0.003033332255461629</v>
       </c>
       <c r="G14">
-        <v>0.07693738093256641</v>
+        <v>2.226070835053252</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>YJU2</t>
+          <t>CLIP2</t>
         </is>
       </c>
       <c r="B15">
-        <v>9.396666666666668</v>
+        <v>1.036202796042748</v>
       </c>
       <c r="C15">
-        <v>21.09122222222222</v>
+        <v>3.41983769021339</v>
       </c>
       <c r="D15">
-        <v>5.014086967567523</v>
+        <v>5.753791950959098</v>
       </c>
       <c r="E15">
-        <v>0.0002092682419034496</v>
+        <v>8.426192348044535E-05</v>
       </c>
       <c r="F15">
-        <v>0.04057478690239107</v>
+        <v>0.00393147209821864</v>
       </c>
       <c r="G15">
-        <v>-0.1160010882512967</v>
+        <v>1.721976404009241</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CD9</t>
+          <t>IGLV3.21</t>
         </is>
       </c>
       <c r="B16">
-        <v>7.301000000000001</v>
+        <v>2.460230004339163</v>
       </c>
       <c r="C16">
-        <v>16.02216666666667</v>
+        <v>6.88231010570504</v>
       </c>
       <c r="D16">
-        <v>4.97088602513279</v>
+        <v>5.548510657354591</v>
       </c>
       <c r="E16">
-        <v>0.0002263493406607563</v>
+        <v>0.000117180654924911</v>
       </c>
       <c r="F16">
-        <v>0.04125725724704012</v>
+        <v>0.005006688200885763</v>
       </c>
       <c r="G16">
-        <v>-0.1628126270505525</v>
+        <v>1.393096311907704</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NDUFB5</t>
+          <t>IGLV5.37</t>
         </is>
       </c>
       <c r="B17">
-        <v>9.557666666666679</v>
+        <v>1.81980027020783</v>
       </c>
       <c r="C17">
-        <v>35.10694444444445</v>
+        <v>3.376902268663281</v>
       </c>
       <c r="D17">
-        <v>4.920298966837091</v>
+        <v>5.427847715016521</v>
       </c>
       <c r="E17">
-        <v>0.000248207150789727</v>
+        <v>0.0001426402904104433</v>
       </c>
       <c r="F17">
-        <v>0.04283468271440363</v>
+        <v>0.005580881317628331</v>
       </c>
       <c r="G17">
-        <v>-0.2180636597474015</v>
+        <v>1.196874465707634</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HIGD1A</t>
+          <t>JPT1</t>
         </is>
       </c>
       <c r="B18">
-        <v>4.367333333333332</v>
+        <v>1.34786983271779</v>
       </c>
       <c r="C18">
-        <v>15.10316666666667</v>
+        <v>5.097068135599605</v>
       </c>
       <c r="D18">
-        <v>4.839056435851185</v>
+        <v>5.073618873480056</v>
       </c>
       <c r="E18">
-        <v>0.0002880099373976273</v>
+        <v>0.0002570512057591727</v>
       </c>
       <c r="F18">
-        <v>0.0454448462213867</v>
+        <v>0.00795309138386093</v>
       </c>
       <c r="G18">
-        <v>-0.3077781499728403</v>
+        <v>0.6086412074599936</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PSMC1</t>
+          <t>IGHG2</t>
         </is>
       </c>
       <c r="B19">
-        <v>13.73466666666667</v>
+        <v>1.288419460661124</v>
       </c>
       <c r="C19">
-        <v>51.91283333333334</v>
+        <v>7.878590581879838</v>
       </c>
       <c r="D19">
-        <v>4.827794057312586</v>
+        <v>5.052201296640828</v>
       </c>
       <c r="E19">
-        <v>0.0002940291676439971</v>
+        <v>0.0002665183135747208</v>
       </c>
       <c r="F19">
-        <v>0.0454448462213867</v>
+        <v>0.008027596692543899</v>
       </c>
       <c r="G19">
-        <v>-0.3203101855451091</v>
+        <v>0.5725048089381435</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HERPUD1</t>
+          <t>IGLC1</t>
         </is>
       </c>
       <c r="B20">
-        <v>118.5956666666666</v>
+        <v>1.163471164072827</v>
       </c>
       <c r="C20">
-        <v>389.9133333333334</v>
+        <v>9.65067217159068</v>
       </c>
       <c r="D20">
-        <v>4.803130539497948</v>
+        <v>4.871578585860106</v>
       </c>
       <c r="E20">
-        <v>0.0003076708118769547</v>
+        <v>0.0003624741171235344</v>
       </c>
       <c r="F20">
-        <v>0.0454448462213867</v>
+        <v>0.009642032536289142</v>
       </c>
       <c r="G20">
-        <v>-0.3478348879164228</v>
+        <v>0.2652507998892784</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ZFP36L1</t>
+          <t>IGLV3.10</t>
         </is>
       </c>
       <c r="B21">
-        <v>48.34166666666668</v>
+        <v>1.18958263674525</v>
       </c>
       <c r="C21">
-        <v>151.2787222222222</v>
+        <v>6.450100520976612</v>
       </c>
       <c r="D21">
-        <v>4.714842977855798</v>
+        <v>4.711328724823684</v>
       </c>
       <c r="E21">
-        <v>0.0003621261321156885</v>
+        <v>0.0004779263202987984</v>
       </c>
       <c r="F21">
-        <v>0.04650509057669638</v>
+        <v>0.01097343985422899</v>
       </c>
       <c r="G21">
-        <v>-0.4472702986493085</v>
+        <v>-0.01098371526208108</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LRRC42</t>
+          <t>MCRIP2</t>
         </is>
       </c>
       <c r="B22">
-        <v>1.614333333333333</v>
+        <v>1.088654873160709</v>
       </c>
       <c r="C22">
-        <v>5.607277777777778</v>
+        <v>3.463683213230454</v>
       </c>
       <c r="D22">
-        <v>4.656770884955058</v>
+        <v>4.096421084342348</v>
       </c>
       <c r="E22">
-        <v>0.0004033084751969674</v>
+        <v>0.001423016732932746</v>
       </c>
       <c r="F22">
-        <v>0.04933763213838036</v>
+        <v>0.01955247400761922</v>
       </c>
       <c r="G22">
-        <v>-0.5134426549355045</v>
+        <v>-1.099179218809211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>